<commit_message>
vault backup: 2026-01-19 09:22:19
</commit_message>
<xml_diff>
--- a/BWL/Übung/Prüfung_Übung/UE12_KPIs_19.1.Abgabe/KPIs_Analyse.xlsx
+++ b/BWL/Übung/Prüfung_Übung/UE12_KPIs_19.1.Abgabe/KPIs_Analyse.xlsx
@@ -3,13 +3,156 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11985"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+  <si>
+    <t>EK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lf Verb.</t>
+  </si>
+  <si>
+    <t>Kf.Verb</t>
+  </si>
+  <si>
+    <t>AV</t>
+  </si>
+  <si>
+    <t>UV</t>
+  </si>
+  <si>
+    <t>FK</t>
+  </si>
+  <si>
+    <t>a)</t>
+  </si>
+  <si>
+    <t>Eigenkapitalquote:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EK / GK * 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EK =</t>
+  </si>
+  <si>
+    <t>GK</t>
+  </si>
+  <si>
+    <t>b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anlagendeckung (Grad II)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(EK + langfr. Verbindl.)/AV</t>
+  </si>
+  <si>
+    <t>c)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verschuldungsgrad (statisch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FK / EK</t>
+  </si>
+  <si>
+    <t>d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liquidität Grad I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kassa, Bank / kf. Verb</t>
+  </si>
+  <si>
+    <t>e)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liquidität Grad 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Cash + Forderungen)/kf. Verb</t>
+  </si>
+  <si>
+    <t>f)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kurzfr. UV - kurzfr. Verb.</t>
+  </si>
+  <si>
+    <t>g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liquidität Grad 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ges. UV / Verbindl.</t>
+  </si>
+  <si>
+    <t>h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operativer Cashflow</t>
+  </si>
+  <si>
+    <t>Effektivverschuldung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fremdkap - alles liquide</t>
+  </si>
+  <si>
+    <t>i)</t>
+  </si>
+  <si>
+    <t>Schuldentilgungsdauer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effektivverschuldung / Cashflow</t>
+  </si>
+  <si>
+    <t>j)</t>
+  </si>
+  <si>
+    <t>Eigenkapitalrentabilität</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gewinn / Eigenkapital</t>
+  </si>
+  <si>
+    <t>k)</t>
+  </si>
+  <si>
+    <t>Gesamtkapitalrentabilität</t>
+  </si>
+  <si>
+    <t>(Gewinn+FKZinsen)/(EK+FK)</t>
+  </si>
+  <si>
+    <t>I)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umschlagshäufigkeit des Vermögens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz / GesKap</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -32,18 +175,25 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -59,6 +209,136 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>314324</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>81776</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4387331" cy="2349002"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1962078393" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="923924" y="257036"/>
+          <a:ext cx="4387331" cy="2349002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>447674</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>105119</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705224" cy="1152180"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1959990710" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId2"/>
+        <a:srcRect l="0" t="0" r="0" b="20294"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="1057274" y="2558759"/>
+          <a:ext cx="3705224" cy="1152180"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>314324</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>83819</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3962359" cy="2284094"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1689857361" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="923924" y="6393179"/>
+          <a:ext cx="3962359" cy="2284094"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>314324</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>41909</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3552824" cy="1024111"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2139841319" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="923924" y="8980169"/>
+          <a:ext cx="3552824" cy="1024111"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -387,74 +667,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -462,7 +682,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -488,7 +708,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -565,7 +785,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -601,7 +821,356 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="2" ht="14.25">
+      <c r="B2" s="1"/>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="J3">
+        <v>150</v>
+      </c>
+      <c r="K3">
+        <v>200</v>
+      </c>
+      <c r="L3">
+        <v>100</v>
+      </c>
+      <c r="M3">
+        <v>350</v>
+      </c>
+      <c r="N3">
+        <v>100</v>
+      </c>
+      <c r="O3">
+        <f>K3+L3</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="J7" t="s">
+        <v>6</v>
+      </c>
+      <c r="K7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="K8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N8">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="M9" t="s">
+        <v>10</v>
+      </c>
+      <c r="N9">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="K10">
+        <f>(N8/N9)*100</f>
+        <v>33.333333333333329</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="J12" t="s">
+        <v>11</v>
+      </c>
+      <c r="K12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="K14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="K15">
+        <f>(J3+K3)/M3*100</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="J16" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="B17" s="1"/>
+      <c r="K17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="K18">
+        <f>O3/J3*100</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="J19" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="K21">
+        <f>20/L3*100</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="J22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="K23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="K24">
+        <f>50/L3*100</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="J25" t="s">
+        <v>23</v>
+      </c>
+      <c r="K25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="K26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="K27">
+        <f>(100-100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="J28" t="s">
+        <v>26</v>
+      </c>
+      <c r="K28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="K29" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="K30">
+        <f>100/100*100</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="J35" t="s">
+        <v>0</v>
+      </c>
+      <c r="K35" t="s">
+        <v>1</v>
+      </c>
+      <c r="L35" t="s">
+        <v>2</v>
+      </c>
+      <c r="M35" t="s">
+        <v>3</v>
+      </c>
+      <c r="N35" t="s">
+        <v>4</v>
+      </c>
+      <c r="O35" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="B36" s="1"/>
+      <c r="J36" s="3">
+        <v>150</v>
+      </c>
+      <c r="K36" s="3">
+        <v>200</v>
+      </c>
+      <c r="L36" s="3">
+        <v>100</v>
+      </c>
+      <c r="M36" s="3">
+        <v>350</v>
+      </c>
+      <c r="N36" s="3">
+        <v>100</v>
+      </c>
+      <c r="O36" s="3">
+        <f>K36+L36</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="J40" t="s">
+        <v>29</v>
+      </c>
+      <c r="K40" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="K41">
+        <f>20+30+40</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="K43">
+        <f>800-450-250-10</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="K45" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="K46" t="s">
+        <v>32</v>
+      </c>
+      <c r="N46">
+        <f>O36-20</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="B48" s="1"/>
+      <c r="J48" t="s">
+        <v>33</v>
+      </c>
+      <c r="K48" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" ht="14.25">
+      <c r="K49" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" ht="14.25">
+      <c r="K50">
+        <f>N46/90</f>
+        <v>3.1111111111111112</v>
+      </c>
+    </row>
+    <row r="53" ht="14.25">
+      <c r="J53" t="s">
+        <v>36</v>
+      </c>
+      <c r="K53" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" ht="14.25">
+      <c r="K54" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" ht="14.25">
+      <c r="K55">
+        <f>20/J36*100</f>
+        <v>13.333333333333334</v>
+      </c>
+    </row>
+    <row r="58" ht="14.25">
+      <c r="J58" t="s">
+        <v>39</v>
+      </c>
+      <c r="K58" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59" ht="14.25">
+      <c r="K59" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" ht="14.25">
+      <c r="K60">
+        <f>30/450*100</f>
+        <v>6.666666666666667</v>
+      </c>
+    </row>
+    <row r="62" ht="14.25">
+      <c r="J62" t="s">
+        <v>42</v>
+      </c>
+      <c r="K62" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="K63" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="K64">
+        <f>800/450</f>
+        <v>1.7777777777777777</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>